<commit_message>
ajusta na etiqueta vermelha
</commit_message>
<xml_diff>
--- a/doc/Banco de dados - Falhas.xlsx
+++ b/doc/Banco de dados - Falhas.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\E841371\Documents\Projetos\BR92_Cadastro_Falhas\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\E841371\Documents\Projetos\cadastro_falhas\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1F1DF35-2A6C-4424-B16A-5F75BC52BA68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B74A851-D01C-4E40-8C21-90D20DB5D6BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="44880" yWindow="-6210" windowWidth="16440" windowHeight="28320" firstSheet="1" activeTab="4" xr2:uid="{D4CEC219-B88B-4EB2-9705-7AF54EC3DD85}"/>
   </bookViews>
@@ -1353,7 +1353,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="11">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1361,14 +1361,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF00"/>
-          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1512,7 +1504,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5A3D0D2E-AAE2-4148-A575-DB6FDA85C242}" name="Table1" displayName="Table1" ref="A4:B114" totalsRowShown="0" headerRowDxfId="11" tableBorderDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5A3D0D2E-AAE2-4148-A575-DB6FDA85C242}" name="Table1" displayName="Table1" ref="A4:B114" totalsRowShown="0" headerRowDxfId="10" tableBorderDxfId="9">
   <autoFilter ref="A4:B114" xr:uid="{820131BD-CF24-49C6-AEAC-D27D105AD100}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{85B66FE1-CE0A-4A95-BEE0-AB88518549C8}" name="LINHA"/>
@@ -1523,26 +1515,26 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F78AFC5C-4B55-491E-B82A-15379767E8C5}" name="Table24" displayName="Table24" ref="A1:B104" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F78AFC5C-4B55-491E-B82A-15379767E8C5}" name="Table24" displayName="Table24" ref="A1:B104" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
   <autoFilter ref="A1:B104" xr:uid="{F78AFC5C-4B55-491E-B82A-15379767E8C5}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B84">
     <sortCondition ref="A2:A84"/>
   </sortState>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{B567CB55-C429-4396-8ECD-77DF75DCF725}" name="DESCRIÇÃO DA FALHA" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{EFA4E7EA-444C-4DF5-BAA2-978F84C2DFFF}" name="Família" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{B567CB55-C429-4396-8ECD-77DF75DCF725}" name="DESCRIÇÃO DA FALHA" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{EFA4E7EA-444C-4DF5-BAA2-978F84C2DFFF}" name="Família" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{818FE281-472E-49E8-9FEB-925E5434452A}" name="Table5" displayName="Table5" ref="F1:H36" totalsRowShown="0" headerRowDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{818FE281-472E-49E8-9FEB-925E5434452A}" name="Table5" displayName="Table5" ref="F1:H36" totalsRowShown="0" headerRowDxfId="4">
   <autoFilter ref="F1:H36" xr:uid="{818FE281-472E-49E8-9FEB-925E5434452A}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{766B01AB-4F0A-4F5D-9E42-8F472CF6ACD7}" name="DESCRIÇÃO DA FALHA" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{6BA0409E-098A-4A72-A5B4-523B625F5F97}" name="Família" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{F64274ED-B1DC-42CD-A1E2-34584FE397CF}" name="Status" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{766B01AB-4F0A-4F5D-9E42-8F472CF6ACD7}" name="DESCRIÇÃO DA FALHA" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{6BA0409E-098A-4A72-A5B4-523B625F5F97}" name="Família" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{F64274ED-B1DC-42CD-A1E2-34584FE397CF}" name="Status" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4079,7 +4071,6 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1397F712-BBE8-4688-AF2E-B593A59C2F61}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:C135"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4098,7 +4089,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="2" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="40" t="s">
         <v>137</v>
       </c>
@@ -4106,31 +4097,31 @@
         <v>154</v>
       </c>
     </row>
-    <row r="3" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="40"/>
       <c r="B3" s="9" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="4" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="40"/>
       <c r="B4" s="9" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="5" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="40"/>
       <c r="B5" s="9" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="6" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="40"/>
       <c r="B6" s="9" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="7" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="40"/>
       <c r="B7" s="9" t="s">
         <v>151</v>
@@ -4163,103 +4154,103 @@
         <v>257</v>
       </c>
     </row>
-    <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="40"/>
       <c r="B11" s="9" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="12" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="40"/>
       <c r="B12" s="9" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="13" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="40"/>
       <c r="B13" s="9" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="14" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="40"/>
       <c r="B14" s="9" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="40"/>
       <c r="B15" s="9" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="16" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="40"/>
       <c r="B16" s="9" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="17" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="40"/>
       <c r="B17" s="9" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="18" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="40"/>
       <c r="B18" s="9" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="19" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="40"/>
       <c r="B19" s="9" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="20" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="40"/>
       <c r="B20" s="9" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="21" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="40"/>
       <c r="B21" s="9" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="22" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="40"/>
       <c r="B22" s="9" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="23" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="40"/>
       <c r="B23" s="9" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="24" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="40"/>
       <c r="B24" s="9" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="25" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="40"/>
       <c r="B25" s="9" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="26" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="40"/>
       <c r="B26" s="11" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="27" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="40" t="s">
         <v>221</v>
       </c>
@@ -4267,109 +4258,109 @@
         <v>162</v>
       </c>
     </row>
-    <row r="28" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="40"/>
       <c r="B28" s="9" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="29" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="40"/>
       <c r="B29" s="9" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="30" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="40"/>
       <c r="B30" s="9" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="31" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="40"/>
       <c r="B31" s="9" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="32" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="40"/>
       <c r="B32" s="9" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="33" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="40"/>
       <c r="B33" s="9" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="34" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="40"/>
       <c r="B34" s="9" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="35" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="40"/>
       <c r="B35" s="9" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="36" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="40"/>
       <c r="B36" s="9" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="37" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="40"/>
       <c r="B37" s="10" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="38" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="40"/>
       <c r="B38" s="9" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="39" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="40"/>
       <c r="B39" s="9" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="40" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="40"/>
       <c r="B40" s="9" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="41" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="40"/>
       <c r="B41" s="9" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="42" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="40"/>
       <c r="B42" s="9" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="43" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="40"/>
       <c r="B43" s="9" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="44" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="40"/>
       <c r="B44" s="9" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="45" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="40"/>
       <c r="B45" s="9" t="s">
         <v>214</v>
@@ -4384,13 +4375,13 @@
         <v>257</v>
       </c>
     </row>
-    <row r="47" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="40"/>
       <c r="B47" s="9" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="48" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="40"/>
       <c r="B48" s="9" t="s">
         <v>158</v>
@@ -4405,7 +4396,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="50" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="40"/>
       <c r="B50" s="9" t="s">
         <v>209</v>
@@ -4420,25 +4411,25 @@
         <v>257</v>
       </c>
     </row>
-    <row r="52" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="40"/>
       <c r="B52" s="9" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="53" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="40"/>
       <c r="B53" s="9" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="54" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="40"/>
       <c r="B54" s="11" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="55" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="40" t="s">
         <v>220</v>
       </c>
@@ -4446,25 +4437,25 @@
         <v>157</v>
       </c>
     </row>
-    <row r="56" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="40"/>
       <c r="B56" s="9" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="57" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="40"/>
       <c r="B57" s="9" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="58" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="40"/>
       <c r="B58" s="9" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="59" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="40"/>
       <c r="B59" s="9" t="s">
         <v>167</v>
@@ -4479,175 +4470,175 @@
         <v>259</v>
       </c>
     </row>
-    <row r="61" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" s="40"/>
       <c r="B61" s="9" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="62" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="40"/>
       <c r="B62" s="9" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="63" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" s="40"/>
       <c r="B63" s="9" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="64" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" s="40"/>
       <c r="B64" s="9" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="65" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="40"/>
       <c r="B65" s="9" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="66" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" s="40"/>
       <c r="B66" s="9" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="67" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" s="40"/>
       <c r="B67" s="9" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="68" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" s="40"/>
       <c r="B68" s="9" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="69" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" s="40"/>
       <c r="B69" s="9" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="70" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" s="40"/>
       <c r="B70" s="9" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="71" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" s="40"/>
       <c r="B71" s="9" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="72" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" s="40"/>
       <c r="B72" s="9" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="73" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" s="40"/>
       <c r="B73" s="9" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="74" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" s="40"/>
       <c r="B74" s="9" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="75" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" s="40"/>
       <c r="B75" s="9" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="76" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" s="40"/>
       <c r="B76" s="9" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="77" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" s="40"/>
       <c r="B77" s="9" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="78" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" s="40"/>
       <c r="B78" s="9" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="79" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" s="40"/>
       <c r="B79" s="9" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="80" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" s="40"/>
       <c r="B80" s="9" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="81" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" s="40"/>
       <c r="B81" s="9" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="82" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" s="40"/>
       <c r="B82" s="9" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="83" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" s="40"/>
       <c r="B83" s="9" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="84" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" s="40"/>
       <c r="B84" s="9" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="85" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" s="40"/>
       <c r="B85" s="9" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="86" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" s="40"/>
       <c r="B86" s="9" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="87" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" s="40"/>
       <c r="B87" s="9" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="88" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" s="40"/>
       <c r="B88" s="9" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="89" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" s="40"/>
       <c r="B89" s="9" t="s">
         <v>192</v>
@@ -4662,13 +4653,13 @@
         <v>257</v>
       </c>
     </row>
-    <row r="91" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" s="40"/>
       <c r="B91" s="9" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="92" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" s="40"/>
       <c r="B92" s="9" t="s">
         <v>158</v>
@@ -4683,7 +4674,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="94" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" s="40"/>
       <c r="B94" s="9" t="s">
         <v>209</v>
@@ -4698,49 +4689,49 @@
         <v>257</v>
       </c>
     </row>
-    <row r="96" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" s="40"/>
       <c r="B96" s="9" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="97" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" s="40"/>
       <c r="B97" s="9" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="98" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" s="40"/>
       <c r="B98" s="9" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="99" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" s="40"/>
       <c r="B99" s="9" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="100" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" s="40"/>
       <c r="B100" s="9" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="101" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" s="40"/>
       <c r="B101" s="9" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="102" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" s="40"/>
       <c r="B102" s="11" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="103" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" s="40" t="s">
         <v>109</v>
       </c>
@@ -4748,43 +4739,43 @@
         <v>156</v>
       </c>
     </row>
-    <row r="104" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" s="40"/>
       <c r="B104" s="9" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="105" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" s="40"/>
       <c r="B105" s="9" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="106" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" s="40"/>
       <c r="B106" s="9" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="107" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" s="40"/>
       <c r="B107" s="9" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="108" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" s="40"/>
       <c r="B108" s="9" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="109" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" s="40"/>
       <c r="B109" s="9" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="110" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" s="40"/>
       <c r="B110" s="9" t="s">
         <v>159</v>
@@ -4799,13 +4790,13 @@
         <v>257</v>
       </c>
     </row>
-    <row r="112" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" s="40"/>
       <c r="B112" s="9" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="113" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" s="40"/>
       <c r="B113" s="9" t="s">
         <v>158</v>
@@ -4820,7 +4811,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="115" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" s="40"/>
       <c r="B115" s="9" t="s">
         <v>209</v>
@@ -4835,19 +4826,19 @@
         <v>257</v>
       </c>
     </row>
-    <row r="117" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" s="40"/>
       <c r="B117" s="9" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="118" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" s="40"/>
       <c r="B118" s="11" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="119" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" s="40" t="s">
         <v>222</v>
       </c>
@@ -4855,31 +4846,31 @@
         <v>156</v>
       </c>
     </row>
-    <row r="120" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" s="40"/>
       <c r="B120" s="9" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="121" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" s="40"/>
       <c r="B121" s="9" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="122" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" s="40"/>
       <c r="B122" s="9" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="123" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" s="40"/>
       <c r="B123" s="9" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="124" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" s="40"/>
       <c r="B124" s="9" t="s">
         <v>159</v>
@@ -4894,19 +4885,19 @@
         <v>257</v>
       </c>
     </row>
-    <row r="126" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" s="40"/>
       <c r="B126" s="9" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="127" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" s="40"/>
       <c r="B127" s="9" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="128" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" s="40"/>
       <c r="B128" s="9" t="s">
         <v>209</v>
@@ -4921,13 +4912,13 @@
         <v>257</v>
       </c>
     </row>
-    <row r="130" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" s="40"/>
       <c r="B130" s="9" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="131" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" s="40"/>
       <c r="B131" s="11" t="s">
         <v>176</v>
@@ -4972,11 +4963,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C135" xr:uid="{1397F712-BBE8-4688-AF2E-B593A59C2F61}">
-    <filterColumn colId="1">
-      <colorFilter dxfId="1"/>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:C135" xr:uid="{1397F712-BBE8-4688-AF2E-B593A59C2F61}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B132:B135">
     <sortCondition ref="B132:B135"/>
   </sortState>

</xml_diff>